<commit_message>
removed solve before constraint
</commit_message>
<xml_diff>
--- a/doc/RTL_Bug_Tracking.xlsx
+++ b/doc/RTL_Bug_Tracking.xlsx
@@ -527,9 +527,6 @@
     <t>RTL_012</t>
   </si>
   <si>
-    <t>17/9/2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">
 TX - Half Duplex -Collision</t>
   </si>
@@ -554,6 +551,9 @@
   <si>
     <t xml:space="preserve">1058268213
 </t>
+  </si>
+  <si>
+    <t>17/8/2026</t>
   </si>
 </sst>
 </file>
@@ -1562,7 +1562,7 @@
         <v>137</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H12" s="24" t="s">
         <v>22</v>
@@ -1592,7 +1592,7 @@
         <v>143</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="C13" s="26" t="s">
         <v>30</v>
@@ -1601,22 +1601,22 @@
         <v>72</v>
       </c>
       <c r="E13" s="28" t="s">
+        <v>144</v>
+      </c>
+      <c r="F13" s="29" t="s">
         <v>145</v>
       </c>
-      <c r="F13" s="29" t="s">
-        <v>146</v>
-      </c>
       <c r="G13" s="30" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H13" s="24" t="s">
         <v>64</v>
       </c>
       <c r="I13" s="26" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J13" s="28" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K13" s="16" t="s">
         <v>55</v>
@@ -1625,10 +1625,10 @@
         <v>86</v>
       </c>
       <c r="M13" s="30" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="N13" s="26" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O13" s="30" t="s">
         <v>115</v>

</xml_diff>